<commit_message>
Mark required fields in the forms and the bulk template
Forms: required fields carry a red * (hidden from screen readers, which
read the required attribute) and each form says '* Required' once at the
top. The property form's Ownership becomes Tenure, required, matching the
rest of the app and the template; the details panel says Tenure too.

Template: two clear heading tiers, required in deep teal with a *,
optional in pale teal; required columns are tinted pale yellow all the way
down; their cell hints start with 'Required'; the Instructions sheet says
Required or Optional for every column.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/templates/property-bulk-upload-template.xlsx
+++ b/docs/templates/property-bulk-upload-template.xlsx
@@ -71,7 +71,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -93,6 +93,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE3F7F6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF4CE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -118,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -142,6 +148,11 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -153,11 +164,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="1" max="1" width="30" customWidth="1" style="12"/>
     <col min="2" max="2" width="16" customWidth="1" style="3"/>
-    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1" style="12"/>
     <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="24" customWidth="1"/>
+    <col min="5" max="5" width="24" customWidth="1" style="12"/>
     <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="7" width="20" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
@@ -166,8 +177,8 @@
     <col min="11" max="11" width="16" customWidth="1"/>
     <col min="12" max="12" width="16" customWidth="1"/>
     <col min="13" max="13" width="12" customWidth="1" style="3"/>
-    <col min="14" max="14" width="12" customWidth="1" style="9"/>
-    <col min="15" max="15" width="12" customWidth="1" style="9"/>
+    <col min="14" max="14" width="12" customWidth="1" style="13"/>
+    <col min="15" max="15" width="12" customWidth="1" style="13"/>
     <col min="16" max="16" width="12" customWidth="1"/>
     <col min="17" max="17" width="15" customWidth="1"/>
     <col min="18" max="18" width="13" customWidth="1"/>
@@ -191,7 +202,7 @@
           <t>Property name *</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr" s="1">
+      <c r="B1" t="inlineStr" s="11">
         <is>
           <t>Property code</t>
         </is>
@@ -201,7 +212,7 @@
           <t>Property type *</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr" s="1">
+      <c r="D1" t="inlineStr" s="11">
         <is>
           <t>Owning company</t>
         </is>
@@ -211,42 +222,42 @@
           <t>Tenure *</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr" s="1">
+      <c r="F1" t="inlineStr" s="11">
         <is>
           <t>Structure</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr" s="1">
+      <c r="G1" t="inlineStr" s="11">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr" s="1">
+      <c r="H1" t="inlineStr" s="11">
         <is>
           <t>Location code</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr" s="1">
+      <c r="I1" t="inlineStr" s="11">
         <is>
           <t>Address line 1</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr" s="1">
+      <c r="J1" t="inlineStr" s="11">
         <is>
           <t>Address line 2</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr" s="1">
+      <c r="K1" t="inlineStr" s="11">
         <is>
           <t>City / town</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr" s="1">
+      <c r="L1" t="inlineStr" s="11">
         <is>
           <t>District</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr" s="1">
+      <c r="M1" t="inlineStr" s="11">
         <is>
           <t>Postal code</t>
         </is>
@@ -261,77 +272,77 @@
           <t>Longitude *</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr" s="1">
+      <c r="P1" t="inlineStr" s="11">
         <is>
           <t>Land extent</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr" s="1">
+      <c r="Q1" t="inlineStr" s="11">
         <is>
           <t>Land unit</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr" s="1">
+      <c r="R1" t="inlineStr" s="11">
         <is>
           <t>Building area</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr" s="1">
+      <c r="S1" t="inlineStr" s="11">
         <is>
           <t>Building unit</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr" s="1">
+      <c r="T1" t="inlineStr" s="11">
         <is>
           <t>Assessment no.</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr" s="1">
+      <c r="U1" t="inlineStr" s="11">
         <is>
           <t>Survey plan no.</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr" s="1">
+      <c r="V1" t="inlineStr" s="11">
         <is>
           <t>Lot no.</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr" s="1">
+      <c r="W1" t="inlineStr" s="11">
         <is>
           <t>Acquisition date</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr" s="1">
+      <c r="X1" t="inlineStr" s="11">
         <is>
           <t>Acquisition cost</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr" s="1">
+      <c r="Y1" t="inlineStr" s="11">
         <is>
           <t>Current value</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr" s="1">
+      <c r="Z1" t="inlineStr" s="11">
         <is>
           <t>Currency</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr" s="1">
+      <c r="AA1" t="inlineStr" s="11">
         <is>
           <t>Current use</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr" s="1">
+      <c r="AB1" t="inlineStr" s="11">
         <is>
           <t>Custodian / officer</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr" s="1">
+      <c r="AC1" t="inlineStr" s="11">
         <is>
           <t>Contact phone</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr" s="1">
+      <c r="AD1" t="inlineStr" s="11">
         <is>
           <t>Notes</t>
         </is>
@@ -340,15 +351,15 @@
   </sheetData>
   <autoFilter ref="A1:AD1"/>
   <dataValidations count="30">
-    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Property name" prompt="The property's name as people know it, e.g. Kandy City Showroom." sqref="A2:A2001"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Property name (required)" prompt="Required. The property's name as people know it, e.g. Kandy City Showroom." sqref="A2:A2001"/>
     <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Property code" prompt="Leave blank to generate one from the property type (e.g. COMM-0004). Must be unique." sqref="B2:B2001"/>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" showInputMessage="1" promptTitle="Property type" prompt="What the property is used for. Pick from the list." errorTitle="Not in the list" error="Choose a value from the drop-down list." sqref="C2:C2001">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" showInputMessage="1" promptTitle="Property type (required)" prompt="Required. What the property is used for. Pick from the list." errorTitle="Not in the list" error="Choose a value from the drop-down list." sqref="C2:C2001">
       <formula1>lst_types</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" showInputMessage="1" promptTitle="Owning company" prompt="Short code of the group company holding title. Leave blank if leased or rented in." errorTitle="Not in the list" error="Choose a value from the drop-down list." sqref="D2:D2001">
       <formula1>lst_entities</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" showInputMessage="1" promptTitle="Tenure" prompt="How the property is held. Pick from the list." errorTitle="Not in the list" error="Choose a value from the drop-down list." sqref="E2:E2001">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" showInputMessage="1" promptTitle="Tenure (required)" prompt="Required. How the property is held. Pick from the list." errorTitle="Not in the list" error="Choose a value from the drop-down list." sqref="E2:E2001">
       <formula1>lst_tenures</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" showInputMessage="1" promptTitle="Structure" prompt="Bare land, Land &amp; building or Building only. Blank means Land &amp; building." errorTitle="Not in the list" error="Choose a value from the drop-down list." sqref="F2:F2001">
@@ -367,11 +378,11 @@
       <formula1>lst_districts</formula1>
     </dataValidation>
     <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Postal code" prompt="Postal code." sqref="M2:M2001"/>
-    <dataValidation type="decimal" operator="between" allowBlank="1" showErrorMessage="1" showInputMessage="1" promptTitle="Latitude" prompt="Decimal degrees, e.g. 7.293600. Can be left blank if a location code with coordinates is given." errorTitle="Outside Sri Lanka" error="Latitude must be between 5.8 and 9.95." sqref="N2:N2001">
+    <dataValidation type="decimal" operator="between" allowBlank="1" showErrorMessage="1" showInputMessage="1" promptTitle="Latitude (required)" prompt="Required. Decimal degrees, e.g. 7.293600. Can be left blank if a location code with coordinates is given." errorTitle="Outside Sri Lanka" error="Latitude must be between 5.8 and 9.95." sqref="N2:N2001">
       <formula1>5.8</formula1>
       <formula2>9.95</formula2>
     </dataValidation>
-    <dataValidation type="decimal" operator="between" allowBlank="1" showErrorMessage="1" showInputMessage="1" promptTitle="Longitude" prompt="Decimal degrees, e.g. 80.635100. Can be left blank if a location code with coordinates is given." errorTitle="Outside Sri Lanka" error="Longitude must be between 79.4 and 82.05." sqref="O2:O2001">
+    <dataValidation type="decimal" operator="between" allowBlank="1" showErrorMessage="1" showInputMessage="1" promptTitle="Longitude (required)" prompt="Required. Decimal degrees, e.g. 80.635100. Can be left blank if a location code with coordinates is given." errorTitle="Outside Sri Lanka" error="Longitude must be between 79.4 and 82.05." sqref="O2:O2001">
       <formula1>79.4</formula1>
       <formula2>82.05</formula2>
     </dataValidation>
@@ -432,7 +443,7 @@
     <row r="3" ht="34" customHeight="1">
       <c r="A3" t="inlineStr" s="6">
         <is>
-          <t>1. Keep the headings in row 1 as they are. Columns marked * are required; the dark headings mark them.</t>
+          <t>1. Keep the headings in row 1 as they are. Required columns have a dark heading with a * and pale yellow cells: fill those in for every property. Light headings are optional.</t>
         </is>
       </c>
     </row>
@@ -484,12 +495,12 @@
     <row r="10">
       <c r="A10" t="inlineStr" s="10">
         <is>
-          <t>Property name</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr" s="6">
-        <is>
-          <t>Yes</t>
+          <t>Property name *</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr" s="12">
+        <is>
+          <t>Required</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="6">
@@ -504,7 +515,11 @@
           <t>Property code</t>
         </is>
       </c>
-      <c r="B11" s="6"/>
+      <c r="B11" t="inlineStr" s="6">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
       <c r="C11" t="inlineStr" s="6">
         <is>
           <t>Leave blank to generate one from the property type (e.g. COMM-0004). Must be unique.</t>
@@ -514,12 +529,12 @@
     <row r="12">
       <c r="A12" t="inlineStr" s="10">
         <is>
-          <t>Property type</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr" s="6">
-        <is>
-          <t>Yes</t>
+          <t>Property type *</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr" s="12">
+        <is>
+          <t>Required</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="6">
@@ -534,7 +549,11 @@
           <t>Owning company</t>
         </is>
       </c>
-      <c r="B13" s="6"/>
+      <c r="B13" t="inlineStr" s="6">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
       <c r="C13" t="inlineStr" s="6">
         <is>
           <t>Short code of the group company holding title. Leave blank if leased or rented in. Allowed values: the Owning companies column on the Lists sheet.</t>
@@ -544,12 +563,12 @@
     <row r="14">
       <c r="A14" t="inlineStr" s="10">
         <is>
-          <t>Tenure</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr" s="6">
-        <is>
-          <t>Yes</t>
+          <t>Tenure *</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr" s="12">
+        <is>
+          <t>Required</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="6">
@@ -564,7 +583,11 @@
           <t>Structure</t>
         </is>
       </c>
-      <c r="B15" s="6"/>
+      <c r="B15" t="inlineStr" s="6">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr" s="6">
         <is>
           <t>Bare land, Land &amp; building or Building only. Blank means Land &amp; building. Allowed values: the Structures column on the Lists sheet.</t>
@@ -577,7 +600,11 @@
           <t>Status</t>
         </is>
       </c>
-      <c r="B16" s="6"/>
+      <c r="B16" t="inlineStr" s="6">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
       <c r="C16" t="inlineStr" s="6">
         <is>
           <t>Blank means Active / in use. Allowed values: the Statuses column on the Lists sheet.</t>
@@ -590,7 +617,11 @@
           <t>Location code</t>
         </is>
       </c>
-      <c r="B17" s="6"/>
+      <c r="B17" t="inlineStr" s="6">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr" s="6">
         <is>
           <t>Code from the location master. If coordinates are blank, the property is placed at this location. Allowed values: the Location codes column on the Lists sheet.</t>
@@ -603,7 +634,11 @@
           <t>Address line 1</t>
         </is>
       </c>
-      <c r="B18" s="6"/>
+      <c r="B18" t="inlineStr" s="6">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr" s="6">
         <is>
           <t>Street address.</t>
@@ -616,7 +651,11 @@
           <t>Address line 2</t>
         </is>
       </c>
-      <c r="B19" s="6"/>
+      <c r="B19" t="inlineStr" s="6">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
       <c r="C19" t="inlineStr" s="6">
         <is>
           <t>Optional second address line.</t>
@@ -629,7 +668,11 @@
           <t>City / town</t>
         </is>
       </c>
-      <c r="B20" s="6"/>
+      <c r="B20" t="inlineStr" s="6">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr" s="6">
         <is>
           <t>City or town.</t>
@@ -642,7 +685,11 @@
           <t>District</t>
         </is>
       </c>
-      <c r="B21" s="6"/>
+      <c r="B21" t="inlineStr" s="6">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
       <c r="C21" t="inlineStr" s="6">
         <is>
           <t>One of the 25 districts. The province is filled in for you. Allowed values: the Districts column on the Lists sheet.</t>
@@ -655,7 +702,11 @@
           <t>Postal code</t>
         </is>
       </c>
-      <c r="B22" s="6"/>
+      <c r="B22" t="inlineStr" s="6">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr" s="6">
         <is>
           <t>Postal code.</t>
@@ -665,12 +716,12 @@
     <row r="23">
       <c r="A23" t="inlineStr" s="10">
         <is>
-          <t>Latitude</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr" s="6">
-        <is>
-          <t>Yes</t>
+          <t>Latitude *</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr" s="12">
+        <is>
+          <t>Required</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="6">
@@ -682,12 +733,12 @@
     <row r="24">
       <c r="A24" t="inlineStr" s="10">
         <is>
-          <t>Longitude</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr" s="6">
-        <is>
-          <t>Yes</t>
+          <t>Longitude *</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr" s="12">
+        <is>
+          <t>Required</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="6">
@@ -702,7 +753,11 @@
           <t>Land extent</t>
         </is>
       </c>
-      <c r="B25" s="6"/>
+      <c r="B25" t="inlineStr" s="6">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
       <c r="C25" t="inlineStr" s="6">
         <is>
           <t>Land area as a number, e.g. 42.5.</t>
@@ -715,7 +770,11 @@
           <t>Land unit</t>
         </is>
       </c>
-      <c r="B26" s="6"/>
+      <c r="B26" t="inlineStr" s="6">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
       <c r="C26" t="inlineStr" s="6">
         <is>
           <t>Unit of the land extent. Blank means Perches. Allowed values: the Units column on the Lists sheet.</t>
@@ -728,7 +787,11 @@
           <t>Building area</t>
         </is>
       </c>
-      <c r="B27" s="6"/>
+      <c r="B27" t="inlineStr" s="6">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
       <c r="C27" t="inlineStr" s="6">
         <is>
           <t>Floor area as a number.</t>
@@ -741,7 +804,11 @@
           <t>Building unit</t>
         </is>
       </c>
-      <c r="B28" s="6"/>
+      <c r="B28" t="inlineStr" s="6">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
       <c r="C28" t="inlineStr" s="6">
         <is>
           <t>Unit of the building area. Blank means the same as the land unit. Allowed values: the Units column on the Lists sheet.</t>
@@ -754,7 +821,11 @@
           <t>Assessment no.</t>
         </is>
       </c>
-      <c r="B29" s="6"/>
+      <c r="B29" t="inlineStr" s="6">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
       <c r="C29" t="inlineStr" s="6">
         <is>
           <t>Local authority assessment number.</t>
@@ -767,7 +838,11 @@
           <t>Survey plan no.</t>
         </is>
       </c>
-      <c r="B30" s="6"/>
+      <c r="B30" t="inlineStr" s="6">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
       <c r="C30" t="inlineStr" s="6">
         <is>
           <t>Survey plan number.</t>
@@ -780,7 +855,11 @@
           <t>Lot no.</t>
         </is>
       </c>
-      <c r="B31" s="6"/>
+      <c r="B31" t="inlineStr" s="6">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
       <c r="C31" t="inlineStr" s="6">
         <is>
           <t>Lot number on the plan.</t>
@@ -793,7 +872,11 @@
           <t>Acquisition date</t>
         </is>
       </c>
-      <c r="B32" s="6"/>
+      <c r="B32" t="inlineStr" s="6">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
       <c r="C32" t="inlineStr" s="6">
         <is>
           <t>Date acquired, e.g. 2019-03-31 or 31/03/2019 (day first). An Excel date works too.</t>
@@ -806,7 +889,11 @@
           <t>Acquisition cost</t>
         </is>
       </c>
-      <c r="B33" s="6"/>
+      <c r="B33" t="inlineStr" s="6">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
       <c r="C33" t="inlineStr" s="6">
         <is>
           <t>Amount paid, e.g. 12500000.</t>
@@ -819,7 +906,11 @@
           <t>Current value</t>
         </is>
       </c>
-      <c r="B34" s="6"/>
+      <c r="B34" t="inlineStr" s="6">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
       <c r="C34" t="inlineStr" s="6">
         <is>
           <t>Latest value, e.g. 18000000.</t>
@@ -832,7 +923,11 @@
           <t>Currency</t>
         </is>
       </c>
-      <c r="B35" s="6"/>
+      <c r="B35" t="inlineStr" s="6">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
       <c r="C35" t="inlineStr" s="6">
         <is>
           <t>Blank means LKR.</t>
@@ -845,7 +940,11 @@
           <t>Current use</t>
         </is>
       </c>
-      <c r="B36" s="6"/>
+      <c r="B36" t="inlineStr" s="6">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
       <c r="C36" t="inlineStr" s="6">
         <is>
           <t>What the property is used for today.</t>
@@ -858,7 +957,11 @@
           <t>Custodian / officer</t>
         </is>
       </c>
-      <c r="B37" s="6"/>
+      <c r="B37" t="inlineStr" s="6">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
       <c r="C37" t="inlineStr" s="6">
         <is>
           <t>The person responsible for it.</t>
@@ -871,7 +974,11 @@
           <t>Contact phone</t>
         </is>
       </c>
-      <c r="B38" s="6"/>
+      <c r="B38" t="inlineStr" s="6">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
       <c r="C38" t="inlineStr" s="6">
         <is>
           <t>Phone number for the site or custodian.</t>
@@ -884,7 +991,11 @@
           <t>Notes</t>
         </is>
       </c>
-      <c r="B39" s="6"/>
+      <c r="B39" t="inlineStr" s="6">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
       <c r="C39" t="inlineStr" s="6">
         <is>
           <t>Anything else worth recording.</t>
@@ -908,11 +1019,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="1" max="1" width="30" customWidth="1" style="12"/>
+    <col min="2" max="2" width="16" customWidth="1" style="3"/>
+    <col min="3" max="3" width="28" customWidth="1" style="12"/>
     <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="24" customWidth="1"/>
+    <col min="5" max="5" width="24" customWidth="1" style="12"/>
     <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="7" width="20" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
@@ -920,23 +1031,23 @@
     <col min="10" max="10" width="20" customWidth="1"/>
     <col min="11" max="11" width="16" customWidth="1"/>
     <col min="12" max="12" width="16" customWidth="1"/>
-    <col min="13" max="13" width="12" customWidth="1"/>
-    <col min="14" max="14" width="12" customWidth="1"/>
-    <col min="15" max="15" width="12" customWidth="1"/>
+    <col min="13" max="13" width="12" customWidth="1" style="3"/>
+    <col min="14" max="14" width="12" customWidth="1" style="13"/>
+    <col min="15" max="15" width="12" customWidth="1" style="13"/>
     <col min="16" max="16" width="12" customWidth="1"/>
     <col min="17" max="17" width="15" customWidth="1"/>
     <col min="18" max="18" width="13" customWidth="1"/>
     <col min="19" max="19" width="15" customWidth="1"/>
-    <col min="20" max="20" width="16" customWidth="1"/>
-    <col min="21" max="21" width="16" customWidth="1"/>
-    <col min="22" max="22" width="10" customWidth="1"/>
-    <col min="23" max="23" width="15" customWidth="1"/>
+    <col min="20" max="20" width="16" customWidth="1" style="3"/>
+    <col min="21" max="21" width="16" customWidth="1" style="3"/>
+    <col min="22" max="22" width="10" customWidth="1" style="3"/>
+    <col min="23" max="23" width="15" customWidth="1" style="4"/>
     <col min="24" max="24" width="16" customWidth="1"/>
     <col min="25" max="25" width="16" customWidth="1"/>
-    <col min="26" max="26" width="10" customWidth="1"/>
+    <col min="26" max="26" width="10" customWidth="1" style="3"/>
     <col min="27" max="27" width="24" customWidth="1"/>
     <col min="28" max="28" width="20" customWidth="1"/>
-    <col min="29" max="29" width="15" customWidth="1"/>
+    <col min="29" max="29" width="15" customWidth="1" style="3"/>
     <col min="30" max="30" width="30" customWidth="1"/>
   </cols>
   <sheetData>
@@ -946,7 +1057,7 @@
           <t>Property name *</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr" s="1">
+      <c r="B1" t="inlineStr" s="11">
         <is>
           <t>Property code</t>
         </is>
@@ -956,7 +1067,7 @@
           <t>Property type *</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr" s="1">
+      <c r="D1" t="inlineStr" s="11">
         <is>
           <t>Owning company</t>
         </is>
@@ -966,42 +1077,42 @@
           <t>Tenure *</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr" s="1">
+      <c r="F1" t="inlineStr" s="11">
         <is>
           <t>Structure</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr" s="1">
+      <c r="G1" t="inlineStr" s="11">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr" s="1">
+      <c r="H1" t="inlineStr" s="11">
         <is>
           <t>Location code</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr" s="1">
+      <c r="I1" t="inlineStr" s="11">
         <is>
           <t>Address line 1</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr" s="1">
+      <c r="J1" t="inlineStr" s="11">
         <is>
           <t>Address line 2</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr" s="1">
+      <c r="K1" t="inlineStr" s="11">
         <is>
           <t>City / town</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr" s="1">
+      <c r="L1" t="inlineStr" s="11">
         <is>
           <t>District</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr" s="1">
+      <c r="M1" t="inlineStr" s="11">
         <is>
           <t>Postal code</t>
         </is>
@@ -1016,90 +1127,90 @@
           <t>Longitude *</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr" s="1">
+      <c r="P1" t="inlineStr" s="11">
         <is>
           <t>Land extent</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr" s="1">
+      <c r="Q1" t="inlineStr" s="11">
         <is>
           <t>Land unit</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr" s="1">
+      <c r="R1" t="inlineStr" s="11">
         <is>
           <t>Building area</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr" s="1">
+      <c r="S1" t="inlineStr" s="11">
         <is>
           <t>Building unit</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr" s="1">
+      <c r="T1" t="inlineStr" s="11">
         <is>
           <t>Assessment no.</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr" s="1">
+      <c r="U1" t="inlineStr" s="11">
         <is>
           <t>Survey plan no.</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr" s="1">
+      <c r="V1" t="inlineStr" s="11">
         <is>
           <t>Lot no.</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr" s="1">
+      <c r="W1" t="inlineStr" s="11">
         <is>
           <t>Acquisition date</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr" s="1">
+      <c r="X1" t="inlineStr" s="11">
         <is>
           <t>Acquisition cost</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr" s="1">
+      <c r="Y1" t="inlineStr" s="11">
         <is>
           <t>Current value</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr" s="1">
+      <c r="Z1" t="inlineStr" s="11">
         <is>
           <t>Currency</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr" s="1">
+      <c r="AA1" t="inlineStr" s="11">
         <is>
           <t>Current use</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr" s="1">
+      <c r="AB1" t="inlineStr" s="11">
         <is>
           <t>Custodian / officer</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr" s="1">
+      <c r="AC1" t="inlineStr" s="11">
         <is>
           <t>Contact phone</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr" s="1">
+      <c r="AD1" t="inlineStr" s="11">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="inlineStr" s="12">
         <is>
           <t>Kandy City Showroom</t>
         </is>
       </c>
       <c r="B2" s="3"/>
-      <c r="C2" t="inlineStr">
+      <c r="C2" t="inlineStr" s="12">
         <is>
           <t>Educational</t>
         </is>
@@ -1109,7 +1220,7 @@
           <t>CNT</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" t="inlineStr" s="12">
         <is>
           <t>Freehold (owned)</t>
         </is>
@@ -1149,10 +1260,10 @@
           <t>20000</t>
         </is>
       </c>
-      <c r="N2" s="9">
+      <c r="N2" s="13">
         <v>7.2936</v>
       </c>
-      <c r="O2" s="9">
+      <c r="O2" s="13">
         <v>80.6413</v>
       </c>
       <c r="P2">
@@ -1224,18 +1335,18 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="inlineStr" s="12">
         <is>
           <t>Galle Hostel</t>
         </is>
       </c>
       <c r="B3" s="3"/>
-      <c r="C3" t="inlineStr">
+      <c r="C3" t="inlineStr" s="12">
         <is>
           <t>Hostels</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" t="inlineStr" s="12">
         <is>
           <t>Rented in</t>
         </is>
@@ -1261,10 +1372,10 @@
         </is>
       </c>
       <c r="M3" s="3"/>
-      <c r="N3" s="9">
+      <c r="N3" s="13">
         <v>6.026</v>
       </c>
-      <c r="O3" s="9">
+      <c r="O3" s="13">
         <v>80.217</v>
       </c>
       <c r="P3">

</xml_diff>